<commit_message>
altmetric ID paper 22
</commit_message>
<xml_diff>
--- a/StatPub/AltMetric.xlsx
+++ b/StatPub/AltMetric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeremycarlot/Documents/Website/JayCrlt.github.io/StatPub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1224601-223A-714A-966F-99826D4185CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D96A9C4-018D-1745-B2A1-2276F6929E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="660" windowWidth="24300" windowHeight="15040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -889,8 +889,11 @@
       <c r="B24" t="s">
         <v>64</v>
       </c>
+      <c r="C24">
+        <v>204056161</v>
+      </c>
       <c r="D24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>